<commit_message>
SBMD-13 test: yeni test verisi (PENTEST260821-26), SBM'de kullanilmamis il/ilce ciftleri
DB temizligi SBM'deki kayitlari silmedigi icin onceki iki testte 2026-8'e
gonderilen 12 il/ilce cifti tekrar kullanilamaz (RISK-HAVUZU-00004). Yeni ciftler
Temmuz 2026 uretim ekstresinden: 9/0, 10/0, 20/0, 2/1182, 2/1989, 3/1200.
Duzeltme dosyasinda PENTEST260822 ve PENTEST260824 +%20. Bruno hedefleri guncellendi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pen Test/test-1-yukleme.xlsx
+++ b/Pen Test/test-1-yukleme.xlsx
@@ -512,7 +512,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -528,26 +528,26 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PENTEST260811</t>
+          <t>PENTEST260821</t>
         </is>
       </c>
       <c r="H2" s="3" t="n">
-        <v>850000</v>
+        <v>720000</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>20000</v>
+        <v>18000</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>83000</v>
+        <v>70200</v>
       </c>
       <c r="L2" t="n">
         <v>10</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>830000</v>
+        <v>702000</v>
       </c>
     </row>
     <row r="3">
@@ -555,7 +555,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -571,26 +571,26 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>PENTEST260811</t>
+          <t>PENTEST260821</t>
         </is>
       </c>
       <c r="H3" s="3" t="n">
-        <v>425000</v>
+        <v>360000</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>10000</v>
+        <v>9000</v>
       </c>
       <c r="J3" t="n">
         <v>2</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>41500</v>
+        <v>35100</v>
       </c>
       <c r="L3" t="n">
         <v>10</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>415000</v>
+        <v>351000</v>
       </c>
     </row>
     <row r="4">
@@ -598,7 +598,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -614,26 +614,26 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PENTEST260812</t>
+          <t>PENTEST260822</t>
         </is>
       </c>
       <c r="H4" s="3" t="n">
-        <v>640000</v>
+        <v>560000</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>62500</v>
+        <v>54800</v>
       </c>
       <c r="L4" t="n">
         <v>10</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>625000</v>
+        <v>548000</v>
       </c>
     </row>
     <row r="5">
@@ -641,7 +641,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -657,26 +657,26 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>PENTEST260812</t>
+          <t>PENTEST260822</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
-        <v>320000</v>
+        <v>280000</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>7500</v>
+        <v>6000</v>
       </c>
       <c r="J5" t="n">
         <v>2</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>31250</v>
+        <v>27400</v>
       </c>
       <c r="L5" t="n">
         <v>10</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>312500</v>
+        <v>274000</v>
       </c>
     </row>
     <row r="6">
@@ -684,7 +684,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -700,26 +700,26 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>PENTEST260813</t>
+          <t>PENTEST260823</t>
         </is>
       </c>
       <c r="H6" s="3" t="n">
-        <v>910000</v>
+        <v>480000</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="J6" t="n">
         <v>1</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>88000</v>
+        <v>47000</v>
       </c>
       <c r="L6" t="n">
         <v>10</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>880000</v>
+        <v>470000</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -743,26 +743,26 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>PENTEST260813</t>
+          <t>PENTEST260823</t>
         </is>
       </c>
       <c r="H7" s="3" t="n">
-        <v>455000</v>
+        <v>240000</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="J7" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>44000</v>
+        <v>23500</v>
       </c>
       <c r="L7" t="n">
         <v>10</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>440000</v>
+        <v>235000</v>
       </c>
     </row>
     <row r="8">
@@ -773,7 +773,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>1246</v>
+        <v>1182</v>
       </c>
       <c r="D8" t="n">
         <v>2320</v>
@@ -786,26 +786,26 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PENTEST260814</t>
+          <t>PENTEST260824</t>
         </is>
       </c>
       <c r="H8" s="3" t="n">
-        <v>45000</v>
+        <v>32000</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>4400</v>
+        <v>3120</v>
       </c>
       <c r="L8" t="n">
         <v>10</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>44000</v>
+        <v>31200</v>
       </c>
     </row>
     <row r="9">
@@ -816,7 +816,7 @@
         <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>1246</v>
+        <v>1182</v>
       </c>
       <c r="D9" t="n">
         <v>2320</v>
@@ -829,26 +829,26 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>PENTEST260814</t>
+          <t>PENTEST260824</t>
         </is>
       </c>
       <c r="H9" s="3" t="n">
-        <v>22500</v>
+        <v>16000</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="J9" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>2200</v>
+        <v>1560</v>
       </c>
       <c r="L9" t="n">
         <v>10</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>22000</v>
+        <v>15600</v>
       </c>
     </row>
     <row r="10">
@@ -859,7 +859,7 @@
         <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>1425</v>
+        <v>1989</v>
       </c>
       <c r="D10" t="n">
         <v>2320</v>
@@ -872,26 +872,26 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>PENTEST260815</t>
+          <t>PENTEST260825</t>
         </is>
       </c>
       <c r="H10" s="3" t="n">
-        <v>28000</v>
+        <v>15000</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>2750</v>
+        <v>1500</v>
       </c>
       <c r="L10" t="n">
         <v>10</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>27500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="11">
@@ -902,7 +902,7 @@
         <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>1425</v>
+        <v>1989</v>
       </c>
       <c r="D11" t="n">
         <v>2320</v>
@@ -915,26 +915,26 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>PENTEST260815</t>
+          <t>PENTEST260825</t>
         </is>
       </c>
       <c r="H11" s="3" t="n">
-        <v>14000</v>
+        <v>7500</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
         <v>2</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>1375</v>
+        <v>750</v>
       </c>
       <c r="L11" t="n">
         <v>10</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>13750</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="12">
@@ -945,7 +945,7 @@
         <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>1281</v>
+        <v>1200</v>
       </c>
       <c r="D12" t="n">
         <v>2320</v>
@@ -958,26 +958,26 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>PENTEST260816</t>
+          <t>PENTEST260826</t>
         </is>
       </c>
       <c r="H12" s="3" t="n">
-        <v>36000</v>
+        <v>41000</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>3540</v>
+        <v>4000</v>
       </c>
       <c r="L12" t="n">
         <v>10</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>35400</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +988,7 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>1281</v>
+        <v>1200</v>
       </c>
       <c r="D13" t="n">
         <v>2320</v>
@@ -1001,26 +1001,26 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>PENTEST260816</t>
+          <t>PENTEST260826</t>
         </is>
       </c>
       <c r="H13" s="3" t="n">
-        <v>18000</v>
+        <v>20500</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J13" t="n">
         <v>2</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>1770</v>
+        <v>2000</v>
       </c>
       <c r="L13" t="n">
         <v>10</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>17700</v>
+        <v>20000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>